<commit_message>
Add SOL income sheet with August MELI
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SOL/MELI/MELI_Conceptos_2026.xlsx
+++ b/SOL/MELI/MELI_Conceptos_2026.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Conceptos por mes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fuentes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ingresos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Conceptos por mes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fuentes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conceptos por mes'!$A$4:$O$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fuentes'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Conceptos por mes'!$A$4:$O$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fuentes'!$A$1:$H$9</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -20,9 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$ARS] #,##0.00;[Red]-[$ARS] #,##0.00;–"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="[$ARS] #,##0.00"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -123,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,6 +157,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -232,6 +241,21 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Cursor</author>
+  </authors>
+  <commentList>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Importe informado: ARS 8.784.847,44. No se proporcionó recibo en esta actualización.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Cursor</author>
@@ -535,6 +559,267 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SOL — Ingresos 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ingresos mensuales de Sol. Los importes se registran según el mes informado y no se mezclan con gastos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>MELI</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Otros ingresos</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="n"/>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26">
+        <f>SUM(B5:C5)</f>
+        <v/>
+      </c>
+      <c r="E5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n"/>
+      <c r="C6" s="26" t="n"/>
+      <c r="D6" s="26">
+        <f>SUM(B6:C6)</f>
+        <v/>
+      </c>
+      <c r="E6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n"/>
+      <c r="C7" s="26" t="n"/>
+      <c r="D7" s="26">
+        <f>SUM(B7:C7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n"/>
+      <c r="C8" s="26" t="n"/>
+      <c r="D8" s="26">
+        <f>SUM(B8:C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n"/>
+      <c r="C9" s="26" t="n"/>
+      <c r="D9" s="26">
+        <f>SUM(B9:C9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="26">
+        <f>SUM(B10:C10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="n"/>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26">
+        <f>SUM(B11:C11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="n">
+        <v>8784847.439999999</v>
+      </c>
+      <c r="C12" s="28" t="n"/>
+      <c r="D12" s="28">
+        <f>SUM(B12:C12)</f>
+        <v/>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>MELI · ingreso neto agosto informado por usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="26">
+        <f>SUM(B13:C13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="26">
+        <f>SUM(B14:C14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+      <c r="D15" s="26">
+        <f>SUM(B15:C15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="n"/>
+      <c r="C16" s="26" t="n"/>
+      <c r="D16" s="26">
+        <f>SUM(B16:C16)</f>
+        <v/>
+      </c>
+      <c r="E16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="B17" s="29">
+        <f>SUM(B5:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="29">
+        <f>SUM(C5:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="29">
+        <f>SUM(D5:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1751,9 +2036,9 @@
   </sheetData>
   <autoFilter ref="A4:O27"/>
   <mergeCells count="4">
-    <mergeCell ref="A2:O2"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A37:O37"/>
+    <mergeCell ref="A2:O2"/>
     <mergeCell ref="A30:O30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1761,7 +2046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Clarify July MELI salary paid in August
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SOL/MELI/MELI_Conceptos_2026.xlsx
+++ b/SOL/MELI/MELI_Conceptos_2026.xlsx
@@ -248,7 +248,7 @@
   <commentList>
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
-        <t>Importe informado: ARS 8.784.847,44. No se proporcionó recibo en esta actualización.</t>
+        <t>ARS 8.784.847,44: sueldo del período julio 2026, cobrado en agosto 2026.</t>
       </text>
     </comment>
   </commentList>
@@ -559,14 +559,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,14 +580,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ingresos mensuales de Sol. Los importes se registran según el mes informado y no se mezclan con gastos.</t>
-        </is>
-      </c>
-    </row>
+          <t>Ingresos por mes de cobro, identificando por separado el período salarial. No se mezclan con gastos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
-          <t>Mes</t>
+          <t>Mes de cobro</t>
         </is>
       </c>
       <c r="B4" s="25" t="inlineStr">
@@ -605,6 +607,11 @@
         </is>
       </c>
       <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Período salarial</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
         <is>
           <t>Comentario</t>
         </is>
@@ -623,6 +630,7 @@
         <v/>
       </c>
       <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -637,6 +645,7 @@
         <v/>
       </c>
       <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -651,6 +660,7 @@
         <v/>
       </c>
       <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -665,6 +675,7 @@
         <v/>
       </c>
       <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -679,6 +690,7 @@
         <v/>
       </c>
       <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -693,6 +705,7 @@
         <v/>
       </c>
       <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -707,6 +720,7 @@
         <v/>
       </c>
       <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
@@ -724,7 +738,12 @@
       </c>
       <c r="E12" s="27" t="inlineStr">
         <is>
-          <t>MELI · ingreso neto agosto informado por usuario</t>
+          <t>Julio 2026</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>MELI · sueldo neto cobrado en agosto</t>
         </is>
       </c>
     </row>
@@ -741,6 +760,7 @@
         <v/>
       </c>
       <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -755,6 +775,7 @@
         <v/>
       </c>
       <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -769,6 +790,7 @@
         <v/>
       </c>
       <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -783,6 +805,7 @@
         <v/>
       </c>
       <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -803,11 +826,12 @@
         <v/>
       </c>
       <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>